<commit_message>
Clean working version: removed NetworkX, legacy flow charts, and ensured only Graphviz Sankey-style diagrams remain
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_scientific.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_scientific.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>iteration</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>S_10_deterministic</t>
+  </si>
+  <si>
+    <t>S_11_deterministic</t>
   </si>
   <si>
     <t>TC_03_04_mc</t>
@@ -407,10 +410,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,8 +450,11 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2">
         <v>0</v>
       </c>
@@ -468,25 +474,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G2">
-        <v>0.3601309695574858</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>0.5732563387720151</v>
+        <v>0.4846642596276388</v>
       </c>
       <c r="I2">
-        <v>0.5585608347956226</v>
+        <v>0.5569390596382893</v>
       </c>
       <c r="J2">
-        <v>0.2171124415507095</v>
+        <v>0.4172473314166346</v>
       </c>
       <c r="K2">
-        <v>0.03177128162947693</v>
+        <v>0.1645401604675616</v>
       </c>
       <c r="L2">
-        <v>0.03048647806881687</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>0.02581553639845666</v>
+      </c>
+      <c r="M2">
+        <v>0.03251838013999736</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3">
         <v>1</v>
       </c>
@@ -506,25 +515,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G3">
-        <v>0.4103077553268482</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>0.5928345522499001</v>
+        <v>0.3163347657747282</v>
       </c>
       <c r="I3">
-        <v>0.5344460245032467</v>
+        <v>0.5542667625456268</v>
       </c>
       <c r="J3">
-        <v>0.2160760717121523</v>
+        <v>0.4819057340995151</v>
       </c>
       <c r="K3">
-        <v>0.03354287954428101</v>
+        <v>0.2236836164751606</v>
       </c>
       <c r="L3">
-        <v>0.0302140937064824</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>0.03225565897555884</v>
+      </c>
+      <c r="M3">
+        <v>0.03631769724358119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4">
         <v>2</v>
       </c>
@@ -544,25 +556,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G4">
-        <v>0.3669715897437242</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>0.5242939946429311</v>
+        <v>0.3840711967620373</v>
       </c>
       <c r="I4">
-        <v>0.4869472778476708</v>
+        <v>0.4720942533734669</v>
       </c>
       <c r="J4">
-        <v>0.2472897943813004</v>
+        <v>0.5267056550281919</v>
       </c>
       <c r="K4">
-        <v>0.01608081568382235</v>
+        <v>0.1640869720167174</v>
       </c>
       <c r="L4">
-        <v>0.03453249743455269</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>0.02354444125566145</v>
+      </c>
+      <c r="M4">
+        <v>0.02819123985061094</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5">
         <v>3</v>
       </c>
@@ -582,25 +597,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G5">
-        <v>0.3198678089868403</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>0.4974167108989428</v>
+        <v>0.3998044883241645</v>
       </c>
       <c r="I5">
-        <v>0.5394753440086411</v>
+        <v>0.5457340599879679</v>
       </c>
       <c r="J5">
-        <v>0.1587730297588421</v>
+        <v>0.4088371669392007</v>
       </c>
       <c r="K5">
-        <v>0.02898482257406015</v>
+        <v>0.1642258940447402</v>
       </c>
       <c r="L5">
-        <v>0.03246425859465748</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>0.02421248855685976</v>
+      </c>
+      <c r="M5">
+        <v>0.0318122263784752</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6">
         <v>4</v>
       </c>
@@ -620,25 +638,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G6">
-        <v>0.4482554068029946</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>0.5367871046800126</v>
+        <v>0.4467217477637678</v>
       </c>
       <c r="I6">
-        <v>0.523848007753433</v>
+        <v>0.4200731382695032</v>
       </c>
       <c r="J6">
-        <v>0.1742133858187908</v>
+        <v>0.4652551522930349</v>
       </c>
       <c r="K6">
-        <v>0.02682800217265861</v>
+        <v>0.1962279265582439</v>
       </c>
       <c r="L6">
-        <v>0.03893372213730634</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>0.0228930723445854</v>
+      </c>
+      <c r="M6">
+        <v>0.02384327013169356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7">
         <v>5</v>
       </c>
@@ -658,25 +679,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G7">
-        <v>0.4582113834235194</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>0.5795251100638237</v>
+        <v>0.3766967955138332</v>
       </c>
       <c r="I7">
-        <v>0.4886858232362418</v>
+        <v>0.5815119972502657</v>
       </c>
       <c r="J7">
-        <v>0.2271355376797713</v>
+        <v>0.4969503842827815</v>
       </c>
       <c r="K7">
-        <v>0.02902441458694776</v>
+        <v>0.2385202011791158</v>
       </c>
       <c r="L7">
-        <v>0.04160798740508818</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>0.02585425554967963</v>
+      </c>
+      <c r="M7">
+        <v>0.03422481476843714</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8">
         <v>6</v>
       </c>
@@ -696,25 +720,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G8">
-        <v>0.4645916004159739</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>0.594203407985467</v>
+        <v>0.4853715110317862</v>
       </c>
       <c r="I8">
-        <v>0.5029063806240796</v>
+        <v>0.4902237793125238</v>
       </c>
       <c r="J8">
-        <v>0.2336421786885101</v>
+        <v>0.4970702409212168</v>
       </c>
       <c r="K8">
-        <v>0.02531791335905556</v>
+        <v>0.1985406507922823</v>
       </c>
       <c r="L8">
-        <v>0.03136211684706132</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>0.02748385050640208</v>
+      </c>
+      <c r="M8">
+        <v>0.03528730590541582</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9">
         <v>7</v>
       </c>
@@ -734,25 +761,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G9">
-        <v>0.4777578039093182</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>0.5152703215588579</v>
+        <v>0.3437323254497998</v>
       </c>
       <c r="I9">
-        <v>0.5820871147996608</v>
+        <v>0.4953763150205728</v>
       </c>
       <c r="J9">
-        <v>0.2249425587242119</v>
+        <v>0.4531791957965875</v>
       </c>
       <c r="K9">
-        <v>0.02380607465490612</v>
+        <v>0.228246411608961</v>
       </c>
       <c r="L9">
-        <v>0.03094710976443618</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>0.02295686751560282</v>
+      </c>
+      <c r="M9">
+        <v>0.03463136309365607</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10">
         <v>8</v>
       </c>
@@ -772,25 +802,28 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G10">
-        <v>0.3907645129063523</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>0.5056745438239194</v>
+        <v>0.405438444720526</v>
       </c>
       <c r="I10">
-        <v>0.5379113756375062</v>
+        <v>0.4316929339890444</v>
       </c>
       <c r="J10">
-        <v>0.1956924049299955</v>
+        <v>0.469947881781668</v>
       </c>
       <c r="K10">
-        <v>0.03116309156033792</v>
+        <v>0.2085744889681235</v>
       </c>
       <c r="L10">
-        <v>0.03495324804531472</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>0.03295898807027421</v>
+      </c>
+      <c r="M10">
+        <v>0.03854492489436261</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11">
         <v>9</v>
       </c>
@@ -810,22 +843,25 @@
         <v>2117.583119837446</v>
       </c>
       <c r="G11">
-        <v>0.3073290060387172</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>0.4590101589791852</v>
+        <v>0.31128016210809</v>
       </c>
       <c r="I11">
-        <v>0.5292406646465868</v>
+        <v>0.4984453226656594</v>
       </c>
       <c r="J11">
-        <v>0.1723350780401522</v>
+        <v>0.4909658327808614</v>
       </c>
       <c r="K11">
-        <v>0.03311351303498275</v>
+        <v>0.1967556403913495</v>
       </c>
       <c r="L11">
-        <v>0.03875542145126092</v>
+        <v>0.0258124241622574</v>
+      </c>
+      <c r="M11">
+        <v>0.03024313007876305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>